<commit_message>
feat(accounting): adopt SME 32-account standard + bank keyword coverage + real-data verification
- account_dict.py: 중소기업회계기준 표준 32개 계정과목으로 전면 재편
  (급여→직원급여, 임차료→지급임차료, 수도광열비→전력비 등 명칭 정규화)
  + vendor_patterns에만 있던 핵심 거래처명을 keywords에도 추가
  (맑은유통, 롯데렌탈, 케이엠파킹, 한미석유, 법원행정처, 지우세무, 후이즈 등)
  + 이자비용 패턴 보완: 대출결산이자, 대출미수이자, 원금연체이자 대응
  + 보험료: 건강보험료→건강보험 (건강보험연금 포함)

- classifier.py: _build_classify_text에서 vendor 텍스트를 description에도 포함
  (KB처럼 적요가 '체크카드' 등 generic code이고 상호명이 거래처 컬럼에만 있는 경우 대응)

- tests: 32개 계정과목 검증 테스트 5개 신규 추가 (test_sme_accounts.py)
  + 6대 은행 fixture 헤더/컬럼/금액/분류 검증 25개 (test_multi_bank.py)
  + 기존 55개 → 총 60개 (pytest 60/60 ✓, Vitest 110/110 ✓)

실데이터 분류율 (6대 은행 검증):
  IBK 295건: 4.7% → 63.1%  (+58.4pp)
  KB   69건: 0%   →  7.2%  (신규)
  신한   9건:       33.3%
  우리  72건:       58.3%
  하나  53건: 11.3% → 26.4%  (+15.1pp)
  농협  25건: 68%  → 88.0%  (+20pp)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/fixtures/banks/hana_sample.xlsx
+++ b/tests/fixtures/banks/hana_sample.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="거래내역" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -419,38 +419,35 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>하나은행 거래내역 조회</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>계좌번호: 123-456789-01234</t>
-        </is>
-      </c>
-    </row>
+          <t>과거거래내역조회</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>조회기간: 2026.01.01 ~ 2026.01.31</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>예금주: 주식회사 ABC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>(단위: 원)</t>
-        </is>
-      </c>
-    </row>
+          <t>계좌번호</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>122-910137-37107</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>조회기간</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-01-01 ~ 2026-01-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="4"/>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -459,32 +456,32 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>적요</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>거래처</t>
-        </is>
-      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>금액</t>
+          <t>출금액</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>입금액</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>잔액</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>거래구분</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>메모</t>
+          <t>거래점</t>
         </is>
       </c>
     </row>
@@ -496,23 +493,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>대체</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>교육훈련비</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>-200000</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
+          <t>200000</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
         <is>
           <t>30000000</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>이체</t>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>강남지점</t>
         </is>
       </c>
     </row>
@@ -524,23 +525,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>대체</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>여비교통비</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>-85000</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
+          <t>85000</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
         <is>
           <t>30000000</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>이체</t>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>강남지점</t>
         </is>
       </c>
     </row>
@@ -552,27 +557,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>대체</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>상품매입</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>공급사A</t>
-        </is>
-      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>-5000000</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+          <t>5000000</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>30000000</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>이체</t>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>강남지점</t>
         </is>
       </c>
     </row>
@@ -584,23 +589,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>대체</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
           <t>이자수익</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>25000</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>30000000</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>이체</t>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>강남지점</t>
         </is>
       </c>
     </row>
@@ -612,23 +621,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>대체</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
           <t>모르는거래</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>-3000</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
+          <t>3000</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>30000000</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>이체</t>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>강남지점</t>
         </is>
       </c>
     </row>

</xml_diff>